<commit_message>
updates in accu table
</commit_message>
<xml_diff>
--- a/Modaliteter/FTV/accu_table.xlsx
+++ b/Modaliteter/FTV/accu_table.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\rvbrtg\Modaliteter\FTV\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44CFE62E-E614-4887-ABB3-CE68725BF1A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94D169B8-A626-4A31-889E-F64BF023EB9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="827" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="830" uniqueCount="20">
   <si>
     <t>Mode</t>
   </si>
@@ -88,6 +88,15 @@
   <si>
     <t>mmAs_per_frame</t>
   </si>
+  <si>
+    <t>bulk</t>
+  </si>
+  <si>
+    <t>gamla barn</t>
+  </si>
+  <si>
+    <t>nya barn?</t>
+  </si>
 </sst>
 </file>
 
@@ -105,12 +114,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -125,10 +140,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -409,12 +428,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K273"/>
+  <dimension ref="A1:M273"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="7.5703125" customWidth="1"/>
     <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="11" max="11" width="17.5703125" customWidth="1"/>
+    <col min="5" max="5" width="3.85546875" customWidth="1"/>
+    <col min="6" max="6" width="4.85546875" customWidth="1"/>
+    <col min="8" max="8" width="5.42578125" customWidth="1"/>
+    <col min="10" max="10" width="7.28515625" customWidth="1"/>
+    <col min="11" max="11" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -2783,7 +2807,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>8</v>
       </c>
@@ -2820,7 +2844,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>8</v>
       </c>
@@ -2857,7 +2881,7 @@
         <v>170.00000000000003</v>
       </c>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>8</v>
       </c>
@@ -2894,7 +2918,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>8</v>
       </c>
@@ -2931,44 +2955,48 @@
         <v>190.00000000000003</v>
       </c>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
-        <v>8</v>
-      </c>
-      <c r="B69">
-        <v>180</v>
-      </c>
-      <c r="C69" s="1">
+    <row r="69" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A69" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B69" s="3">
+        <v>180</v>
+      </c>
+      <c r="C69" s="4">
         <v>5.4</v>
       </c>
-      <c r="D69" t="s">
+      <c r="D69" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E69">
-        <v>85</v>
-      </c>
-      <c r="F69" s="1">
+      <c r="E69" s="3">
+        <v>85</v>
+      </c>
+      <c r="F69" s="4">
         <v>10</v>
       </c>
-      <c r="G69" t="s">
-        <v>7</v>
-      </c>
-      <c r="H69">
+      <c r="G69" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H69" s="3">
         <v>215</v>
       </c>
-      <c r="I69">
+      <c r="I69" s="3">
         <f t="shared" si="2"/>
         <v>54</v>
       </c>
-      <c r="J69">
+      <c r="J69" s="3">
         <v>270</v>
       </c>
-      <c r="K69" s="2">
+      <c r="K69" s="5">
         <f t="shared" si="3"/>
         <v>200</v>
       </c>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L69" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="M69" s="6"/>
+    </row>
+    <row r="70" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>8</v>
       </c>
@@ -3005,7 +3033,7 @@
         <v>34.1796875</v>
       </c>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>8</v>
       </c>
@@ -3042,7 +3070,7 @@
         <v>51.26953125</v>
       </c>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>8</v>
       </c>
@@ -3079,7 +3107,7 @@
         <v>68.359375</v>
       </c>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>8</v>
       </c>
@@ -3116,7 +3144,7 @@
         <v>85.44921875</v>
       </c>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>8</v>
       </c>
@@ -3153,7 +3181,7 @@
         <v>102.5390625</v>
       </c>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>8</v>
       </c>
@@ -3190,7 +3218,7 @@
         <v>119.62890625</v>
       </c>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>8</v>
       </c>
@@ -3227,7 +3255,7 @@
         <v>136.71875</v>
       </c>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>8</v>
       </c>
@@ -3264,7 +3292,7 @@
         <v>153.80859375</v>
       </c>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>8</v>
       </c>
@@ -3301,7 +3329,7 @@
         <v>170.8984375</v>
       </c>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>8</v>
       </c>
@@ -3338,7 +3366,7 @@
         <v>187.98828125</v>
       </c>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>8</v>
       </c>
@@ -3375,7 +3403,7 @@
         <v>205.078125</v>
       </c>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>8</v>
       </c>
@@ -3412,44 +3440,47 @@
         <v>222.16796875</v>
       </c>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
-        <v>8</v>
-      </c>
-      <c r="B82">
-        <v>360</v>
-      </c>
-      <c r="C82" s="1">
+    <row r="82" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A82" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B82" s="3">
+        <v>360</v>
+      </c>
+      <c r="C82" s="4">
         <v>17.5</v>
       </c>
-      <c r="D82" t="s">
+      <c r="D82" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="E82">
-        <v>85</v>
-      </c>
-      <c r="F82" s="1">
-        <v>7</v>
-      </c>
-      <c r="G82" t="s">
-        <v>7</v>
-      </c>
-      <c r="H82">
+      <c r="E82" s="3">
+        <v>85</v>
+      </c>
+      <c r="F82" s="4">
+        <v>7</v>
+      </c>
+      <c r="G82" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H82" s="3">
         <v>489</v>
       </c>
-      <c r="I82">
+      <c r="I82" s="3">
         <f t="shared" si="2"/>
         <v>122.5</v>
       </c>
-      <c r="J82">
+      <c r="J82" s="3">
         <v>512</v>
       </c>
-      <c r="K82" s="2">
+      <c r="K82" s="5">
         <f t="shared" si="3"/>
         <v>239.2578125</v>
       </c>
-    </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L82" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="83" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>8</v>
       </c>
@@ -3486,7 +3517,7 @@
         <v>256.34765625</v>
       </c>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>8</v>
       </c>
@@ -3523,7 +3554,7 @@
         <v>273.4375</v>
       </c>
     </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>8</v>
       </c>
@@ -3560,7 +3591,7 @@
         <v>290.52734375</v>
       </c>
     </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>8</v>
       </c>
@@ -3597,7 +3628,7 @@
         <v>307.6171875</v>
       </c>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>8</v>
       </c>
@@ -3634,7 +3665,7 @@
         <v>324.70703125</v>
       </c>
     </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>8</v>
       </c>
@@ -3671,7 +3702,7 @@
         <v>341.796875</v>
       </c>
     </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>8</v>
       </c>
@@ -3705,7 +3736,7 @@
         <v>33.809001097694839</v>
       </c>
     </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>8</v>
       </c>
@@ -3739,7 +3770,7 @@
         <v>50.713501646542262</v>
       </c>
     </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>8</v>
       </c>
@@ -3773,7 +3804,7 @@
         <v>67.618002195389678</v>
       </c>
     </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>8</v>
       </c>
@@ -3807,7 +3838,7 @@
         <v>84.522502744237102</v>
       </c>
     </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>8</v>
       </c>
@@ -3841,7 +3872,7 @@
         <v>101.42700329308452</v>
       </c>
     </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>8</v>
       </c>
@@ -3875,7 +3906,7 @@
         <v>118.33150384193195</v>
       </c>
     </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>8</v>
       </c>
@@ -3909,7 +3940,7 @@
         <v>135.23600439077936</v>
       </c>
     </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>8</v>
       </c>
@@ -4487,7 +4518,7 @@
         <v>249.19093851132686</v>
       </c>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>8</v>
       </c>
@@ -4521,7 +4552,7 @@
         <v>274.11003236245955</v>
       </c>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>8</v>
       </c>
@@ -4555,7 +4586,7 @@
         <v>299.02912621359224</v>
       </c>
     </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>8</v>
       </c>
@@ -4589,7 +4620,7 @@
         <v>323.94822006472498</v>
       </c>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>8</v>
       </c>
@@ -4623,7 +4654,7 @@
         <v>348.86731391585761</v>
       </c>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>8</v>
       </c>
@@ -4657,7 +4688,7 @@
         <v>373.78640776699029</v>
       </c>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>8</v>
       </c>
@@ -4691,7 +4722,7 @@
         <v>398.70550161812298</v>
       </c>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>8</v>
       </c>
@@ -4712,6 +4743,9 @@
       </c>
       <c r="G119" t="s">
         <v>7</v>
+      </c>
+      <c r="H119">
+        <v>41.9</v>
       </c>
       <c r="I119">
         <f t="shared" si="2"/>
@@ -4725,7 +4759,7 @@
         <v>19.444444444444443</v>
       </c>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>8</v>
       </c>
@@ -4746,6 +4780,9 @@
       </c>
       <c r="G120" t="s">
         <v>7</v>
+      </c>
+      <c r="H120">
+        <v>62.9</v>
       </c>
       <c r="I120">
         <f t="shared" si="2"/>
@@ -4759,7 +4796,7 @@
         <v>29.166666666666668</v>
       </c>
     </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>8</v>
       </c>
@@ -4780,6 +4817,9 @@
       </c>
       <c r="G121" t="s">
         <v>7</v>
+      </c>
+      <c r="H121">
+        <v>83.9</v>
       </c>
       <c r="I121">
         <f t="shared" si="2"/>
@@ -4793,7 +4833,7 @@
         <v>38.888888888888886</v>
       </c>
     </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>8</v>
       </c>
@@ -4814,6 +4854,9 @@
       </c>
       <c r="G122" t="s">
         <v>7</v>
+      </c>
+      <c r="H122">
+        <v>105</v>
       </c>
       <c r="I122">
         <f t="shared" si="2"/>
@@ -4827,7 +4870,7 @@
         <v>48.611111111111114</v>
       </c>
     </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>8</v>
       </c>
@@ -4848,6 +4891,9 @@
       </c>
       <c r="G123" t="s">
         <v>7</v>
+      </c>
+      <c r="H123">
+        <v>126</v>
       </c>
       <c r="I123">
         <f t="shared" si="2"/>
@@ -4861,7 +4907,7 @@
         <v>58.333333333333336</v>
       </c>
     </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>8</v>
       </c>
@@ -4882,6 +4928,9 @@
       </c>
       <c r="G124" t="s">
         <v>7</v>
+      </c>
+      <c r="H124">
+        <v>147</v>
       </c>
       <c r="I124">
         <f t="shared" si="2"/>
@@ -4895,41 +4944,47 @@
         <v>68.055555555555557</v>
       </c>
     </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A125" t="s">
-        <v>8</v>
-      </c>
-      <c r="B125">
-        <v>360</v>
-      </c>
-      <c r="C125" s="1">
+    <row r="125" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A125" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B125" s="3">
+        <v>360</v>
+      </c>
+      <c r="C125" s="4">
         <v>10.5</v>
       </c>
-      <c r="D125" t="s">
+      <c r="D125" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E125">
-        <v>85</v>
-      </c>
-      <c r="F125" s="1">
+      <c r="E125" s="3">
+        <v>85</v>
+      </c>
+      <c r="F125" s="4">
         <v>4</v>
       </c>
-      <c r="G125" t="s">
-        <v>7</v>
-      </c>
-      <c r="I125">
+      <c r="G125" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H125" s="3">
+        <v>168</v>
+      </c>
+      <c r="I125" s="3">
         <f t="shared" si="2"/>
         <v>42</v>
       </c>
-      <c r="J125">
+      <c r="J125" s="3">
         <v>540</v>
       </c>
-      <c r="K125" s="2">
+      <c r="K125" s="5">
         <f t="shared" si="3"/>
         <v>77.777777777777771</v>
       </c>
-    </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L125" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="126" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>8</v>
       </c>
@@ -4950,6 +5005,9 @@
       </c>
       <c r="G126" t="s">
         <v>7</v>
+      </c>
+      <c r="H126">
+        <v>189</v>
       </c>
       <c r="I126">
         <f t="shared" si="2"/>
@@ -4963,7 +5021,7 @@
         <v>87.5</v>
       </c>
     </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>8</v>
       </c>
@@ -4984,6 +5042,9 @@
       </c>
       <c r="G127" t="s">
         <v>7</v>
+      </c>
+      <c r="H127">
+        <v>210</v>
       </c>
       <c r="I127">
         <f t="shared" si="2"/>
@@ -4997,7 +5058,7 @@
         <v>97.222222222222229</v>
       </c>
     </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>8</v>
       </c>
@@ -5018,6 +5079,9 @@
       </c>
       <c r="G128" t="s">
         <v>7</v>
+      </c>
+      <c r="H128">
+        <v>231</v>
       </c>
       <c r="I128">
         <f t="shared" si="2"/>
@@ -5053,6 +5117,9 @@
       <c r="G129" t="s">
         <v>7</v>
       </c>
+      <c r="H129">
+        <v>252</v>
+      </c>
       <c r="I129">
         <f t="shared" si="2"/>
         <v>63</v>
@@ -5087,6 +5154,9 @@
       <c r="G130" t="s">
         <v>7</v>
       </c>
+      <c r="H130">
+        <v>273</v>
+      </c>
       <c r="I130">
         <f t="shared" si="2"/>
         <v>68.25</v>
@@ -5121,6 +5191,9 @@
       <c r="G131" t="s">
         <v>7</v>
       </c>
+      <c r="H131">
+        <v>294</v>
+      </c>
       <c r="I131">
         <f t="shared" ref="I131:I137" si="4">C131*F131</f>
         <v>73.5</v>
@@ -5155,6 +5228,9 @@
       <c r="G132" t="s">
         <v>7</v>
       </c>
+      <c r="H132">
+        <v>315</v>
+      </c>
       <c r="I132">
         <f t="shared" si="4"/>
         <v>78.75</v>
@@ -5189,6 +5265,9 @@
       <c r="G133" t="s">
         <v>7</v>
       </c>
+      <c r="H133">
+        <v>336</v>
+      </c>
       <c r="I133">
         <f t="shared" si="4"/>
         <v>84</v>
@@ -5223,6 +5302,9 @@
       <c r="G134" t="s">
         <v>7</v>
       </c>
+      <c r="H134">
+        <v>358</v>
+      </c>
       <c r="I134">
         <f t="shared" si="4"/>
         <v>89.25</v>
@@ -5257,6 +5339,9 @@
       <c r="G135" t="s">
         <v>7</v>
       </c>
+      <c r="H135">
+        <v>378</v>
+      </c>
       <c r="I135">
         <f t="shared" si="4"/>
         <v>94.5</v>
@@ -5291,6 +5376,9 @@
       <c r="G136" t="s">
         <v>7</v>
       </c>
+      <c r="H136">
+        <v>399</v>
+      </c>
       <c r="I136">
         <f t="shared" si="4"/>
         <v>99.75</v>
@@ -5325,6 +5413,9 @@
       <c r="G137" t="s">
         <v>7</v>
       </c>
+      <c r="H137">
+        <v>419</v>
+      </c>
       <c r="I137">
         <f t="shared" si="4"/>
         <v>105</v>
@@ -10219,38 +10310,38 @@
       </c>
     </row>
     <row r="273" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A273" t="s">
-        <v>8</v>
-      </c>
-      <c r="B273">
-        <v>360</v>
-      </c>
-      <c r="C273" s="1">
+      <c r="A273" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B273" s="3">
+        <v>360</v>
+      </c>
+      <c r="C273" s="4">
         <v>10.5</v>
       </c>
-      <c r="D273" t="s">
+      <c r="D273" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E273">
-        <v>90</v>
-      </c>
-      <c r="F273" s="1">
+      <c r="E273" s="3">
+        <v>90</v>
+      </c>
+      <c r="F273" s="4">
         <v>10</v>
       </c>
-      <c r="G273" t="s">
-        <v>7</v>
-      </c>
-      <c r="H273">
+      <c r="G273" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H273" s="3">
         <v>476</v>
       </c>
-      <c r="I273">
+      <c r="I273" s="3">
         <f t="shared" si="10"/>
         <v>105</v>
       </c>
-      <c r="J273">
+      <c r="J273" s="3">
         <v>540</v>
       </c>
-      <c r="K273" s="2">
+      <c r="K273" s="5">
         <f t="shared" si="11"/>
         <v>194.44444444444446</v>
       </c>

</xml_diff>